<commit_message>
Daily recap, matchup updates, learning and research 2026-08-28
</commit_message>
<xml_diff>
--- a/data/k-props/2026-08-28.xlsx
+++ b/data/k-props/2026-08-28.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="97">
   <si>
     <t>date</t>
   </si>
@@ -145,6 +145,9 @@
     <t>lineup_unweighted_30d_posted</t>
   </si>
   <si>
+    <t>O</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
@@ -154,6 +157,9 @@
     <t>David Peterson</t>
   </si>
   <si>
+    <t>W</t>
+  </si>
+  <si>
     <t>6-7</t>
   </si>
   <si>
@@ -169,10 +175,16 @@
     <t>Opener / bullpen game</t>
   </si>
   <si>
+    <t>L</t>
+  </si>
+  <si>
     <t>Eury Pérez</t>
   </si>
   <si>
     <t>Miami Marlins @ Washington Nationals</t>
+  </si>
+  <si>
+    <t>U</t>
   </si>
   <si>
     <t>Michael Wacha</t>
@@ -871,17 +883,23 @@
       <c r="Y2">
         <v>0.9439</v>
       </c>
+      <c r="Z2">
+        <v>5</v>
+      </c>
       <c r="AA2" t="s">
         <v>44</v>
       </c>
+      <c r="AB2">
+        <v>0.02</v>
+      </c>
       <c r="AC2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD2">
         <v>3.28</v>
       </c>
       <c r="AE2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF2">
         <v>0.1649</v>
@@ -891,6 +909,18 @@
       </c>
       <c r="AH2">
         <v>0.24</v>
+      </c>
+      <c r="AI2">
+        <v>1.72</v>
+      </c>
+      <c r="AJ2">
+        <v>1.72</v>
+      </c>
+      <c r="AK2">
+        <v>1.48</v>
+      </c>
+      <c r="AL2">
+        <v>1.48</v>
       </c>
       <c r="AM2">
         <v>3.52</v>
@@ -901,7 +931,7 @@
         <v>39</v>
       </c>
       <c r="B3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C3">
         <v>4.5</v>
@@ -972,17 +1002,23 @@
       <c r="Y3">
         <v>1.0713</v>
       </c>
+      <c r="Z3">
+        <v>6</v>
+      </c>
       <c r="AA3" t="s">
         <v>44</v>
       </c>
+      <c r="AB3">
+        <v>1.19</v>
+      </c>
       <c r="AC3" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD3">
         <v>6.27</v>
       </c>
       <c r="AE3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="AF3">
         <v>0.2167</v>
@@ -992,6 +1028,18 @@
       </c>
       <c r="AH3">
         <v>-0.58</v>
+      </c>
+      <c r="AI3">
+        <v>-0.27</v>
+      </c>
+      <c r="AJ3">
+        <v>0.27</v>
+      </c>
+      <c r="AK3">
+        <v>0.31</v>
+      </c>
+      <c r="AL3">
+        <v>0.31</v>
       </c>
       <c r="AM3">
         <v>5.69</v>
@@ -1002,7 +1050,7 @@
         <v>39</v>
       </c>
       <c r="B4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C4">
         <v>6.5</v>
@@ -1014,7 +1062,7 @@
         <v>130</v>
       </c>
       <c r="F4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G4">
         <v>824231</v>
@@ -1073,17 +1121,23 @@
       <c r="Y4">
         <v>0.9941</v>
       </c>
+      <c r="Z4">
+        <v>7</v>
+      </c>
       <c r="AA4" t="s">
         <v>44</v>
       </c>
+      <c r="AB4">
+        <v>-0.37</v>
+      </c>
       <c r="AC4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD4">
         <v>6.71</v>
       </c>
       <c r="AE4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="AF4">
         <v>0.3016</v>
@@ -1093,6 +1147,18 @@
       </c>
       <c r="AH4">
         <v>-0.58</v>
+      </c>
+      <c r="AI4">
+        <v>0.29</v>
+      </c>
+      <c r="AJ4">
+        <v>0.29</v>
+      </c>
+      <c r="AK4">
+        <v>0.87</v>
+      </c>
+      <c r="AL4">
+        <v>0.87</v>
       </c>
       <c r="AM4">
         <v>6.13</v>
@@ -1103,7 +1169,7 @@
         <v>39</v>
       </c>
       <c r="B5" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C5">
         <v>4.5</v>
@@ -1115,13 +1181,13 @@
         <v>-120</v>
       </c>
       <c r="F5" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G5">
         <v>824231</v>
       </c>
       <c r="H5" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="I5">
         <v>3</v>
@@ -1174,17 +1240,23 @@
       <c r="Y5">
         <v>0.971</v>
       </c>
+      <c r="Z5">
+        <v>5</v>
+      </c>
       <c r="AA5" t="s">
         <v>44</v>
       </c>
+      <c r="AB5">
+        <v>-1.36</v>
+      </c>
       <c r="AC5" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="AD5">
         <v>2.9</v>
       </c>
       <c r="AE5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF5">
         <v>0.2444</v>
@@ -1194,6 +1266,18 @@
       </c>
       <c r="AH5">
         <v>0.24</v>
+      </c>
+      <c r="AI5">
+        <v>2.1</v>
+      </c>
+      <c r="AJ5">
+        <v>2.1</v>
+      </c>
+      <c r="AK5">
+        <v>1.86</v>
+      </c>
+      <c r="AL5">
+        <v>1.86</v>
       </c>
       <c r="AM5">
         <v>3.14</v>
@@ -1204,7 +1288,7 @@
         <v>39</v>
       </c>
       <c r="B6" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C6">
         <v>5.5</v>
@@ -1216,7 +1300,7 @@
         <v>-111</v>
       </c>
       <c r="F6" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="G6">
         <v>822691</v>
@@ -1275,17 +1359,23 @@
       <c r="Y6">
         <v>1.0228</v>
       </c>
+      <c r="Z6">
+        <v>5</v>
+      </c>
       <c r="AA6" t="s">
-        <v>44</v>
+        <v>57</v>
+      </c>
+      <c r="AB6">
+        <v>0.16</v>
       </c>
       <c r="AC6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD6">
         <v>6.24</v>
       </c>
       <c r="AE6" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="AF6">
         <v>0.2665</v>
@@ -1295,6 +1385,18 @@
       </c>
       <c r="AH6">
         <v>-0.58</v>
+      </c>
+      <c r="AI6">
+        <v>-1.24</v>
+      </c>
+      <c r="AJ6">
+        <v>1.24</v>
+      </c>
+      <c r="AK6">
+        <v>-0.66</v>
+      </c>
+      <c r="AL6">
+        <v>0.66</v>
       </c>
       <c r="AM6">
         <v>5.66</v>
@@ -1305,7 +1407,7 @@
         <v>39</v>
       </c>
       <c r="B7" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="C7">
         <v>4.5</v>
@@ -1317,7 +1419,7 @@
         <v>-160</v>
       </c>
       <c r="F7" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="G7">
         <v>824396</v>
@@ -1376,17 +1478,23 @@
       <c r="Y7">
         <v>0.88</v>
       </c>
+      <c r="Z7">
+        <v>10</v>
+      </c>
       <c r="AA7" t="s">
         <v>44</v>
       </c>
+      <c r="AB7">
+        <v>-0.83</v>
+      </c>
       <c r="AC7" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="AD7">
         <v>3.43</v>
       </c>
       <c r="AE7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF7">
         <v>0.1884</v>
@@ -1396,6 +1504,18 @@
       </c>
       <c r="AH7">
         <v>0.24</v>
+      </c>
+      <c r="AI7">
+        <v>6.57</v>
+      </c>
+      <c r="AJ7">
+        <v>6.57</v>
+      </c>
+      <c r="AK7">
+        <v>6.33</v>
+      </c>
+      <c r="AL7">
+        <v>6.33</v>
       </c>
       <c r="AM7">
         <v>3.67</v>
@@ -1406,7 +1526,7 @@
         <v>39</v>
       </c>
       <c r="B8" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C8">
         <v>4.5</v>
@@ -1418,7 +1538,7 @@
         <v>106</v>
       </c>
       <c r="F8" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="G8">
         <v>824396</v>
@@ -1477,17 +1597,23 @@
       <c r="Y8">
         <v>0.9542</v>
       </c>
+      <c r="Z8">
+        <v>5</v>
+      </c>
       <c r="AA8" t="s">
         <v>44</v>
       </c>
+      <c r="AB8">
+        <v>-0.64</v>
+      </c>
       <c r="AC8" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD8">
         <v>3.62</v>
       </c>
       <c r="AE8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF8">
         <v>0.1976</v>
@@ -1497,6 +1623,18 @@
       </c>
       <c r="AH8">
         <v>0.24</v>
+      </c>
+      <c r="AI8">
+        <v>1.38</v>
+      </c>
+      <c r="AJ8">
+        <v>1.38</v>
+      </c>
+      <c r="AK8">
+        <v>1.14</v>
+      </c>
+      <c r="AL8">
+        <v>1.14</v>
       </c>
       <c r="AM8">
         <v>3.86</v>
@@ -1507,7 +1645,7 @@
         <v>39</v>
       </c>
       <c r="B9" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="C9">
         <v>5.5</v>
@@ -1519,7 +1657,7 @@
         <v>-135</v>
       </c>
       <c r="F9" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="G9">
         <v>823583</v>
@@ -1578,17 +1716,23 @@
       <c r="Y9">
         <v>0.947</v>
       </c>
+      <c r="Z9">
+        <v>10</v>
+      </c>
       <c r="AA9" t="s">
         <v>44</v>
       </c>
+      <c r="AB9">
+        <v>-0.42</v>
+      </c>
       <c r="AC9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD9">
         <v>4.84</v>
       </c>
       <c r="AE9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF9">
         <v>0.2357</v>
@@ -1598,6 +1742,18 @@
       </c>
       <c r="AH9">
         <v>0.24</v>
+      </c>
+      <c r="AI9">
+        <v>5.16</v>
+      </c>
+      <c r="AJ9">
+        <v>5.16</v>
+      </c>
+      <c r="AK9">
+        <v>4.92</v>
+      </c>
+      <c r="AL9">
+        <v>4.92</v>
       </c>
       <c r="AM9">
         <v>5.08</v>
@@ -1608,7 +1764,7 @@
         <v>39</v>
       </c>
       <c r="B10" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="C10">
         <v>5.5</v>
@@ -1620,7 +1776,7 @@
         <v>140</v>
       </c>
       <c r="F10" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="G10">
         <v>823583</v>
@@ -1679,17 +1835,23 @@
       <c r="Y10">
         <v>0.9963</v>
       </c>
+      <c r="Z10">
+        <v>2</v>
+      </c>
       <c r="AA10" t="s">
-        <v>44</v>
+        <v>57</v>
+      </c>
+      <c r="AB10">
+        <v>0.65</v>
       </c>
       <c r="AC10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD10">
         <v>5.91</v>
       </c>
       <c r="AE10" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF10">
         <v>0.2819</v>
@@ -1699,6 +1861,18 @@
       </c>
       <c r="AH10">
         <v>0.24</v>
+      </c>
+      <c r="AI10">
+        <v>-3.91</v>
+      </c>
+      <c r="AJ10">
+        <v>3.91</v>
+      </c>
+      <c r="AK10">
+        <v>-4.15</v>
+      </c>
+      <c r="AL10">
+        <v>4.15</v>
       </c>
       <c r="AM10">
         <v>6.15</v>
@@ -1709,7 +1883,7 @@
         <v>39</v>
       </c>
       <c r="B11" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C11">
         <v>3.5</v>
@@ -1721,7 +1895,7 @@
         <v>110</v>
       </c>
       <c r="F11" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="G11">
         <v>822935</v>
@@ -1780,17 +1954,23 @@
       <c r="Y11">
         <v>0.88</v>
       </c>
+      <c r="Z11">
+        <v>1</v>
+      </c>
       <c r="AA11" t="s">
-        <v>44</v>
+        <v>57</v>
+      </c>
+      <c r="AB11">
+        <v>-0.7</v>
       </c>
       <c r="AC11" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD11">
         <v>2.56</v>
       </c>
       <c r="AE11" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF11">
         <v>0.1931</v>
@@ -1800,6 +1980,18 @@
       </c>
       <c r="AH11">
         <v>0.24</v>
+      </c>
+      <c r="AI11">
+        <v>-1.56</v>
+      </c>
+      <c r="AJ11">
+        <v>1.56</v>
+      </c>
+      <c r="AK11">
+        <v>-1.8</v>
+      </c>
+      <c r="AL11">
+        <v>1.8</v>
       </c>
       <c r="AM11">
         <v>2.8</v>
@@ -1810,7 +2002,7 @@
         <v>39</v>
       </c>
       <c r="B12" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="C12">
         <v>4.5</v>
@@ -1822,7 +2014,7 @@
         <v>-122</v>
       </c>
       <c r="F12" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="G12">
         <v>822935</v>
@@ -1881,17 +2073,23 @@
       <c r="Y12">
         <v>1.028</v>
       </c>
+      <c r="Z12">
+        <v>4</v>
+      </c>
       <c r="AA12" t="s">
-        <v>44</v>
+        <v>57</v>
+      </c>
+      <c r="AB12">
+        <v>-0.24</v>
       </c>
       <c r="AC12" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD12">
         <v>4.02</v>
       </c>
       <c r="AE12" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF12">
         <v>0.2135</v>
@@ -1901,6 +2099,18 @@
       </c>
       <c r="AH12">
         <v>0.24</v>
+      </c>
+      <c r="AI12">
+        <v>-0.02</v>
+      </c>
+      <c r="AJ12">
+        <v>0.02</v>
+      </c>
+      <c r="AK12">
+        <v>-0.26</v>
+      </c>
+      <c r="AL12">
+        <v>0.26</v>
       </c>
       <c r="AM12">
         <v>4.26</v>
@@ -1911,7 +2121,7 @@
         <v>39</v>
       </c>
       <c r="B13" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C13">
         <v>3.5</v>
@@ -1923,7 +2133,7 @@
         <v>-104</v>
       </c>
       <c r="F13" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="G13">
         <v>822769</v>
@@ -1982,17 +2192,23 @@
       <c r="Y13">
         <v>0.9887</v>
       </c>
+      <c r="Z13">
+        <v>1</v>
+      </c>
       <c r="AA13" t="s">
-        <v>44</v>
+        <v>57</v>
+      </c>
+      <c r="AB13">
+        <v>1.28</v>
       </c>
       <c r="AC13" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="AD13">
         <v>4.54</v>
       </c>
       <c r="AE13" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF13">
         <v>0.225</v>
@@ -2002,6 +2218,18 @@
       </c>
       <c r="AH13">
         <v>0.24</v>
+      </c>
+      <c r="AI13">
+        <v>-3.54</v>
+      </c>
+      <c r="AJ13">
+        <v>3.54</v>
+      </c>
+      <c r="AK13">
+        <v>-3.78</v>
+      </c>
+      <c r="AL13">
+        <v>3.78</v>
       </c>
       <c r="AM13">
         <v>4.78</v>
@@ -2012,7 +2240,7 @@
         <v>39</v>
       </c>
       <c r="B14" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C14">
         <v>7.5</v>
@@ -2024,7 +2252,7 @@
         <v>102</v>
       </c>
       <c r="F14" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="G14">
         <v>822769</v>
@@ -2083,17 +2311,23 @@
       <c r="Y14">
         <v>0.9451</v>
       </c>
+      <c r="Z14">
+        <v>8</v>
+      </c>
       <c r="AA14" t="s">
         <v>44</v>
       </c>
+      <c r="AB14">
+        <v>1.12</v>
+      </c>
       <c r="AC14" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD14">
         <v>9.57</v>
       </c>
       <c r="AE14" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="AF14">
         <v>0.3546</v>
@@ -2103,6 +2337,18 @@
       </c>
       <c r="AH14">
         <v>-0.95</v>
+      </c>
+      <c r="AI14">
+        <v>-1.57</v>
+      </c>
+      <c r="AJ14">
+        <v>1.57</v>
+      </c>
+      <c r="AK14">
+        <v>-0.62</v>
+      </c>
+      <c r="AL14">
+        <v>0.62</v>
       </c>
       <c r="AM14">
         <v>8.62</v>
@@ -2113,7 +2359,7 @@
         <v>39</v>
       </c>
       <c r="B15" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C15">
         <v>2.5</v>
@@ -2125,7 +2371,7 @@
         <v>145</v>
       </c>
       <c r="F15" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="G15">
         <v>824877</v>
@@ -2184,17 +2430,23 @@
       <c r="Y15">
         <v>0.9527</v>
       </c>
+      <c r="Z15">
+        <v>4</v>
+      </c>
       <c r="AA15" t="s">
         <v>44</v>
       </c>
+      <c r="AB15">
+        <v>0.91</v>
+      </c>
       <c r="AC15" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD15">
         <v>3.17</v>
       </c>
       <c r="AE15" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF15">
         <v>0.1367</v>
@@ -2204,6 +2456,18 @@
       </c>
       <c r="AH15">
         <v>0.24</v>
+      </c>
+      <c r="AI15">
+        <v>0.83</v>
+      </c>
+      <c r="AJ15">
+        <v>0.83</v>
+      </c>
+      <c r="AK15">
+        <v>0.59</v>
+      </c>
+      <c r="AL15">
+        <v>0.59</v>
       </c>
       <c r="AM15">
         <v>3.41</v>
@@ -2214,7 +2478,7 @@
         <v>39</v>
       </c>
       <c r="B16" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="C16">
         <v>4.5</v>
@@ -2226,7 +2490,7 @@
         <v>-115</v>
       </c>
       <c r="F16" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="G16">
         <v>824877</v>
@@ -2285,17 +2549,23 @@
       <c r="Y16">
         <v>1.0808</v>
       </c>
+      <c r="Z16">
+        <v>3</v>
+      </c>
       <c r="AA16" t="s">
-        <v>44</v>
+        <v>57</v>
+      </c>
+      <c r="AB16">
+        <v>0.64</v>
       </c>
       <c r="AC16" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD16">
         <v>4.9</v>
       </c>
       <c r="AE16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF16">
         <v>0.1785</v>
@@ -2305,6 +2575,18 @@
       </c>
       <c r="AH16">
         <v>0.24</v>
+      </c>
+      <c r="AI16">
+        <v>-1.9</v>
+      </c>
+      <c r="AJ16">
+        <v>1.9</v>
+      </c>
+      <c r="AK16">
+        <v>-2.14</v>
+      </c>
+      <c r="AL16">
+        <v>2.14</v>
       </c>
       <c r="AM16">
         <v>5.14</v>
@@ -2315,7 +2597,7 @@
         <v>39</v>
       </c>
       <c r="B17" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="C17">
         <v>5.5</v>
@@ -2327,7 +2609,7 @@
         <v>-104</v>
       </c>
       <c r="F17" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="G17">
         <v>823504</v>
@@ -2386,17 +2668,23 @@
       <c r="Y17">
         <v>0.9905</v>
       </c>
+      <c r="Z17">
+        <v>7</v>
+      </c>
       <c r="AA17" t="s">
         <v>44</v>
       </c>
+      <c r="AB17">
+        <v>0.62</v>
+      </c>
       <c r="AC17" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD17">
         <v>5.88</v>
       </c>
       <c r="AE17" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF17">
         <v>0.2268</v>
@@ -2406,6 +2694,18 @@
       </c>
       <c r="AH17">
         <v>0.24</v>
+      </c>
+      <c r="AI17">
+        <v>1.12</v>
+      </c>
+      <c r="AJ17">
+        <v>1.12</v>
+      </c>
+      <c r="AK17">
+        <v>0.88</v>
+      </c>
+      <c r="AL17">
+        <v>0.88</v>
       </c>
       <c r="AM17">
         <v>6.12</v>
@@ -2416,7 +2716,7 @@
         <v>39</v>
       </c>
       <c r="B18" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="C18">
         <v>6.5</v>
@@ -2428,7 +2728,7 @@
         <v>104</v>
       </c>
       <c r="F18" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="G18">
         <v>823504</v>
@@ -2487,17 +2787,23 @@
       <c r="Y18">
         <v>1.0264</v>
       </c>
+      <c r="Z18">
+        <v>8</v>
+      </c>
       <c r="AA18" t="s">
         <v>44</v>
       </c>
+      <c r="AB18">
+        <v>-1.08</v>
+      </c>
       <c r="AC18" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="AD18">
         <v>6</v>
       </c>
       <c r="AE18" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="AF18">
         <v>0.3127</v>
@@ -2507,6 +2813,18 @@
       </c>
       <c r="AH18">
         <v>-0.58</v>
+      </c>
+      <c r="AI18">
+        <v>2</v>
+      </c>
+      <c r="AJ18">
+        <v>2</v>
+      </c>
+      <c r="AK18">
+        <v>2.58</v>
+      </c>
+      <c r="AL18">
+        <v>2.58</v>
       </c>
       <c r="AM18">
         <v>5.42</v>
@@ -2517,7 +2835,7 @@
         <v>39</v>
       </c>
       <c r="B19" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="C19">
         <v>3.5</v>
@@ -2529,7 +2847,7 @@
         <v>115</v>
       </c>
       <c r="F19" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="G19">
         <v>823744</v>
@@ -2588,17 +2906,23 @@
       <c r="Y19">
         <v>1.0232</v>
       </c>
+      <c r="Z19">
+        <v>0</v>
+      </c>
       <c r="AA19" t="s">
-        <v>44</v>
+        <v>57</v>
+      </c>
+      <c r="AB19">
+        <v>0.01</v>
       </c>
       <c r="AC19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD19">
         <v>3.27</v>
       </c>
       <c r="AE19" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF19">
         <v>0.1494</v>
@@ -2608,6 +2932,18 @@
       </c>
       <c r="AH19">
         <v>0.24</v>
+      </c>
+      <c r="AI19">
+        <v>-3.27</v>
+      </c>
+      <c r="AJ19">
+        <v>3.27</v>
+      </c>
+      <c r="AK19">
+        <v>-3.51</v>
+      </c>
+      <c r="AL19">
+        <v>3.51</v>
       </c>
       <c r="AM19">
         <v>3.51</v>
@@ -2618,7 +2954,7 @@
         <v>39</v>
       </c>
       <c r="B20" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C20">
         <v>6.5</v>
@@ -2630,7 +2966,7 @@
         <v>-111</v>
       </c>
       <c r="F20" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="G20">
         <v>823744</v>
@@ -2689,17 +3025,23 @@
       <c r="Y20">
         <v>1.0904</v>
       </c>
+      <c r="Z20">
+        <v>7</v>
+      </c>
       <c r="AA20" t="s">
         <v>44</v>
       </c>
+      <c r="AB20">
+        <v>-0.1</v>
+      </c>
       <c r="AC20" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD20">
         <v>7.35</v>
       </c>
       <c r="AE20" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="AF20">
         <v>0.2907</v>
@@ -2709,6 +3051,18 @@
       </c>
       <c r="AH20">
         <v>-0.95</v>
+      </c>
+      <c r="AI20">
+        <v>-0.35</v>
+      </c>
+      <c r="AJ20">
+        <v>0.35</v>
+      </c>
+      <c r="AK20">
+        <v>0.6</v>
+      </c>
+      <c r="AL20">
+        <v>0.6</v>
       </c>
       <c r="AM20">
         <v>6.4</v>
@@ -2719,7 +3073,7 @@
         <v>39</v>
       </c>
       <c r="B21" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="C21">
         <v>3.5</v>
@@ -2731,7 +3085,7 @@
         <v>134</v>
       </c>
       <c r="F21" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="G21">
         <v>823666</v>
@@ -2790,17 +3144,23 @@
       <c r="Y21">
         <v>0.9332</v>
       </c>
+      <c r="Z21">
+        <v>1</v>
+      </c>
       <c r="AA21" t="s">
-        <v>44</v>
+        <v>57</v>
+      </c>
+      <c r="AB21">
+        <v>0.26</v>
       </c>
       <c r="AC21" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD21">
         <v>3.52</v>
       </c>
       <c r="AE21" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF21">
         <v>0.1981</v>
@@ -2810,6 +3170,18 @@
       </c>
       <c r="AH21">
         <v>0.24</v>
+      </c>
+      <c r="AI21">
+        <v>-2.52</v>
+      </c>
+      <c r="AJ21">
+        <v>2.52</v>
+      </c>
+      <c r="AK21">
+        <v>-2.76</v>
+      </c>
+      <c r="AL21">
+        <v>2.76</v>
       </c>
       <c r="AM21">
         <v>3.76</v>
@@ -2820,7 +3192,7 @@
         <v>39</v>
       </c>
       <c r="B22" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="C22">
         <v>5.5</v>
@@ -2832,7 +3204,7 @@
         <v>-138</v>
       </c>
       <c r="F22" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="G22">
         <v>823666</v>
@@ -2891,17 +3263,23 @@
       <c r="Y22">
         <v>1.0791</v>
       </c>
+      <c r="Z22">
+        <v>3</v>
+      </c>
       <c r="AA22" t="s">
-        <v>44</v>
+        <v>57</v>
+      </c>
+      <c r="AB22">
+        <v>0.09</v>
       </c>
       <c r="AC22" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD22">
         <v>6.17</v>
       </c>
       <c r="AE22" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="AF22">
         <v>0.2347</v>
@@ -2911,6 +3289,18 @@
       </c>
       <c r="AH22">
         <v>-0.58</v>
+      </c>
+      <c r="AI22">
+        <v>-3.17</v>
+      </c>
+      <c r="AJ22">
+        <v>3.17</v>
+      </c>
+      <c r="AK22">
+        <v>-2.59</v>
+      </c>
+      <c r="AL22">
+        <v>2.59</v>
       </c>
       <c r="AM22">
         <v>5.59</v>
@@ -2921,7 +3311,7 @@
         <v>39</v>
       </c>
       <c r="B23" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="C23">
         <v>4.5</v>
@@ -2933,7 +3323,7 @@
         <v>115</v>
       </c>
       <c r="F23" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="G23">
         <v>823013</v>
@@ -2992,17 +3382,23 @@
       <c r="Y23">
         <v>0.911</v>
       </c>
+      <c r="Z23">
+        <v>6</v>
+      </c>
       <c r="AA23" t="s">
         <v>44</v>
       </c>
+      <c r="AB23">
+        <v>0.92</v>
+      </c>
       <c r="AC23" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD23">
         <v>5.18</v>
       </c>
       <c r="AE23" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF23">
         <v>0.2534</v>
@@ -3012,6 +3408,18 @@
       </c>
       <c r="AH23">
         <v>0.24</v>
+      </c>
+      <c r="AI23">
+        <v>0.82</v>
+      </c>
+      <c r="AJ23">
+        <v>0.82</v>
+      </c>
+      <c r="AK23">
+        <v>0.58</v>
+      </c>
+      <c r="AL23">
+        <v>0.58</v>
       </c>
       <c r="AM23">
         <v>5.42</v>
@@ -3022,7 +3430,7 @@
         <v>39</v>
       </c>
       <c r="B24" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="C24">
         <v>5.5</v>
@@ -3034,7 +3442,7 @@
         <v>-156</v>
       </c>
       <c r="F24" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="G24">
         <v>823985</v>
@@ -3093,17 +3501,23 @@
       <c r="Y24">
         <v>1.0671</v>
       </c>
+      <c r="Z24">
+        <v>6</v>
+      </c>
       <c r="AA24" t="s">
         <v>44</v>
       </c>
+      <c r="AB24">
+        <v>-0.08</v>
+      </c>
       <c r="AC24" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD24">
         <v>5.18</v>
       </c>
       <c r="AE24" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF24">
         <v>0.2075</v>
@@ -3113,6 +3527,18 @@
       </c>
       <c r="AH24">
         <v>0.24</v>
+      </c>
+      <c r="AI24">
+        <v>0.82</v>
+      </c>
+      <c r="AJ24">
+        <v>0.82</v>
+      </c>
+      <c r="AK24">
+        <v>0.58</v>
+      </c>
+      <c r="AL24">
+        <v>0.58</v>
       </c>
       <c r="AM24">
         <v>5.42</v>
@@ -3123,7 +3549,7 @@
         <v>39</v>
       </c>
       <c r="B25" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="C25">
         <v>6.5</v>
@@ -3135,7 +3561,7 @@
         <v>-102</v>
       </c>
       <c r="F25" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="G25">
         <v>823985</v>
@@ -3194,17 +3620,23 @@
       <c r="Y25">
         <v>0.9462</v>
       </c>
+      <c r="Z25">
+        <v>2</v>
+      </c>
       <c r="AA25" t="s">
-        <v>44</v>
+        <v>57</v>
+      </c>
+      <c r="AB25">
+        <v>-1.13</v>
       </c>
       <c r="AC25" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD25">
         <v>5.13</v>
       </c>
       <c r="AE25" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF25">
         <v>0.3002</v>
@@ -3214,6 +3646,18 @@
       </c>
       <c r="AH25">
         <v>0.24</v>
+      </c>
+      <c r="AI25">
+        <v>-3.13</v>
+      </c>
+      <c r="AJ25">
+        <v>3.13</v>
+      </c>
+      <c r="AK25">
+        <v>-3.37</v>
+      </c>
+      <c r="AL25">
+        <v>3.37</v>
       </c>
       <c r="AM25">
         <v>5.37</v>
@@ -3224,7 +3668,7 @@
         <v>39</v>
       </c>
       <c r="B26" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="C26">
         <v>4.5</v>
@@ -3236,7 +3680,7 @@
         <v>-142</v>
       </c>
       <c r="F26" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="G26">
         <v>824960</v>
@@ -3295,17 +3739,23 @@
       <c r="Y26">
         <v>1.0058</v>
       </c>
+      <c r="Z26">
+        <v>4</v>
+      </c>
       <c r="AA26" t="s">
-        <v>44</v>
+        <v>57</v>
+      </c>
+      <c r="AB26">
+        <v>-0.11</v>
       </c>
       <c r="AC26" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD26">
         <v>4.15</v>
       </c>
       <c r="AE26" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF26">
         <v>0.1797</v>
@@ -3315,6 +3765,18 @@
       </c>
       <c r="AH26">
         <v>0.24</v>
+      </c>
+      <c r="AI26">
+        <v>-0.15</v>
+      </c>
+      <c r="AJ26">
+        <v>0.15</v>
+      </c>
+      <c r="AK26">
+        <v>-0.39</v>
+      </c>
+      <c r="AL26">
+        <v>0.39</v>
       </c>
       <c r="AM26">
         <v>4.39</v>
@@ -3325,7 +3787,7 @@
         <v>39</v>
       </c>
       <c r="B27" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="C27">
         <v>6.5</v>
@@ -3337,7 +3799,7 @@
         <v>-142</v>
       </c>
       <c r="F27" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="G27">
         <v>824960</v>
@@ -3396,17 +3858,23 @@
       <c r="Y27">
         <v>1.116</v>
       </c>
+      <c r="Z27">
+        <v>6</v>
+      </c>
       <c r="AA27" t="s">
-        <v>44</v>
+        <v>57</v>
+      </c>
+      <c r="AB27">
+        <v>-0.19</v>
       </c>
       <c r="AC27" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD27">
         <v>7.26</v>
       </c>
       <c r="AE27" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="AF27">
         <v>0.247</v>
@@ -3416,6 +3884,18 @@
       </c>
       <c r="AH27">
         <v>-0.95</v>
+      </c>
+      <c r="AI27">
+        <v>-1.26</v>
+      </c>
+      <c r="AJ27">
+        <v>1.26</v>
+      </c>
+      <c r="AK27">
+        <v>-0.31</v>
+      </c>
+      <c r="AL27">
+        <v>0.31</v>
       </c>
       <c r="AM27">
         <v>6.31</v>
@@ -3426,16 +3906,16 @@
         <v>39</v>
       </c>
       <c r="B28" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="F28" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="G28">
         <v>823178</v>
       </c>
       <c r="H28" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="I28">
         <v>4.2</v>
@@ -3489,16 +3969,16 @@
         <v>1.0126</v>
       </c>
       <c r="AA28" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC28" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD28">
         <v>3.52</v>
       </c>
       <c r="AE28" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF28">
         <v>0.1688</v>
@@ -3518,10 +3998,10 @@
         <v>39</v>
       </c>
       <c r="B29" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="F29" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="G29">
         <v>823178</v>
@@ -3581,16 +4061,16 @@
         <v>0.88</v>
       </c>
       <c r="AA29" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC29" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD29">
         <v>3.15</v>
       </c>
       <c r="AE29" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF29">
         <v>0.205</v>
@@ -3610,7 +4090,7 @@
         <v>39</v>
       </c>
       <c r="B30" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="C30">
         <v>3.5</v>
@@ -3622,31 +4102,31 @@
         <v>132</v>
       </c>
       <c r="F30" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="G30" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H30" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="L30">
         <v>4</v>
       </c>
       <c r="S30" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="V30" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AA30" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC30" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AE30" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="31" spans="1:39" x14ac:dyDescent="0.25">
@@ -3654,7 +4134,7 @@
         <v>39</v>
       </c>
       <c r="B31" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="C31">
         <v>4.5</v>
@@ -3666,31 +4146,34 @@
         <v>126</v>
       </c>
       <c r="F31" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="G31" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H31" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="L31">
         <v>3</v>
       </c>
       <c r="S31" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="V31" t="s">
-        <v>44</v>
+        <v>45</v>
+      </c>
+      <c r="Z31">
+        <v>7</v>
       </c>
       <c r="AA31" t="s">
         <v>44</v>
       </c>
       <c r="AC31" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AE31" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>